<commit_message>
Update all lod1 metric check
</commit_message>
<xml_diff>
--- a/casebase/statistics/rerord.xlsx
+++ b/casebase/statistics/rerord.xlsx
@@ -1,755 +1,561 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_codes\block-gml-casebase\casebase\statistics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0_code\block-gml-casebase\casebase\statistics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2978715-DFCA-4A56-86AB-89C763AB269D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702EDA43-9577-4C5E-B3CD-C9CAA3382243}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7E148D5C-DE84-49D0-B495-48D3DA96E5A6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="25824" windowHeight="15504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Block" sheetId="3" r:id="rId1"/>
-    <sheet name="LoD1" sheetId="1" r:id="rId2"/>
-    <sheet name="LoD2" sheetId="2" r:id="rId3"/>
+    <sheet name="Block" sheetId="1" r:id="rId1"/>
+    <sheet name="LoD1" sheetId="2" r:id="rId2"/>
+    <sheet name="LoD2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="178">
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>continent</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>data (update) time</t>
+  </si>
+  <si>
+    <t>download time</t>
+  </si>
+  <si>
+    <t>行政区域面积k㎡，只反应osm数据</t>
+  </si>
+  <si>
+    <t>初始切片数量（仅排除&lt;1000）</t>
+  </si>
+  <si>
+    <t>包含lod1的block</t>
+  </si>
+  <si>
+    <t>包含lod2的block</t>
+  </si>
+  <si>
+    <t>简称</t>
+  </si>
+  <si>
+    <t>lod1指标筛除后valid</t>
+  </si>
+  <si>
+    <t>lod2指标筛除后valid</t>
+  </si>
+  <si>
+    <t>总lod1 block</t>
+  </si>
+  <si>
+    <t>总lod2 block</t>
+  </si>
   <si>
     <t>Hamburg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Europe</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>980.23（包含港口海面）</t>
+  </si>
+  <si>
+    <t>DE_HH</t>
+  </si>
+  <si>
+    <t>Vienna</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>AT_VI</t>
+  </si>
+  <si>
+    <t>Amsterdam</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>NL_AM</t>
+  </si>
+  <si>
+    <t>Montreal</t>
+  </si>
+  <si>
+    <t>North America</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>CA_MT</t>
+  </si>
+  <si>
+    <t>Zurich</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>CH_ZU</t>
+  </si>
+  <si>
+    <t>Luxembourg</t>
+  </si>
+  <si>
+    <t>LU_LU</t>
+  </si>
+  <si>
+    <t>Hannover</t>
+  </si>
+  <si>
+    <t>DE_HA</t>
+  </si>
+  <si>
+    <t>Linz</t>
+  </si>
+  <si>
+    <t>AT_LZ</t>
+  </si>
+  <si>
+    <t>Namur</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>BE_NA</t>
+  </si>
+  <si>
+    <t>Prague</t>
+  </si>
+  <si>
+    <t>Czech </t>
+  </si>
+  <si>
+    <t>CZ_PR</t>
+  </si>
+  <si>
+    <t>Dresden</t>
+  </si>
+  <si>
+    <t>DE_DD</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>US_NY</t>
+  </si>
+  <si>
+    <t>Rotterdam </t>
+  </si>
+  <si>
+    <t>NL_RO</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>DE_BE</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>US_SF</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>US_CH</t>
+  </si>
+  <si>
+    <t>Boston</t>
+  </si>
+  <si>
+    <t>US_BO</t>
+  </si>
+  <si>
+    <t>Washington D.C.</t>
+  </si>
+  <si>
+    <t>US_WA</t>
+  </si>
+  <si>
+    <t>Portland</t>
+  </si>
+  <si>
+    <t>US_PO</t>
+  </si>
+  <si>
+    <t>Tokyo</t>
+  </si>
+  <si>
+    <t>Asia</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>42548.04（好多岛）</t>
+  </si>
+  <si>
+    <t>JP_TK</t>
+  </si>
+  <si>
+    <t>Sapporo</t>
+  </si>
+  <si>
+    <t>JP_SP</t>
+  </si>
+  <si>
+    <t>Osaka</t>
+  </si>
+  <si>
+    <t>JP_OS</t>
+  </si>
+  <si>
+    <t>Kanazawa</t>
+  </si>
+  <si>
+    <t>JP_KA</t>
+  </si>
+  <si>
+    <t>Tallinn</t>
+  </si>
+  <si>
+    <t>Estonia</t>
+  </si>
+  <si>
+    <t>EE_TL</t>
+  </si>
+  <si>
+    <t>Toronto</t>
+  </si>
+  <si>
+    <t>CA_TO</t>
+  </si>
+  <si>
+    <t>Winnipeg</t>
+  </si>
+  <si>
+    <t>CA_WP</t>
+  </si>
+  <si>
+    <t>Munich</t>
+  </si>
+  <si>
+    <t>DE_MU</t>
+  </si>
+  <si>
+    <t>Nuremberg</t>
+  </si>
+  <si>
+    <t>DE_NU</t>
+  </si>
+  <si>
+    <t>Beijing</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>CN_BJ</t>
+  </si>
+  <si>
+    <t>Bern</t>
+  </si>
+  <si>
+    <t>CH_BE</t>
+  </si>
+  <si>
+    <t>Bologna</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>IT_BO</t>
+  </si>
+  <si>
+    <t>Lyon</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>FR_LY</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>FR_PA</t>
+  </si>
+  <si>
+    <t>Marseille</t>
+  </si>
+  <si>
+    <t>FR_MA</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>building data source url</t>
+  </si>
+  <si>
+    <t>lod level</t>
+  </si>
+  <si>
+    <t>data time</t>
+  </si>
+  <si>
+    <t>format</t>
+  </si>
+  <si>
+    <t>building count</t>
+  </si>
+  <si>
+    <t>surface count（自建）</t>
+  </si>
+  <si>
+    <t>original SRID</t>
+  </si>
+  <si>
+    <t>匹配到的数量</t>
+  </si>
+  <si>
+    <t>原始数据大小（GB）</t>
+  </si>
+  <si>
+    <t>备注</t>
+  </si>
+  <si>
+    <t>城市数量</t>
+  </si>
+  <si>
+    <t>总building</t>
+  </si>
+  <si>
+    <t>总surface</t>
+  </si>
+  <si>
+    <t>总有效building</t>
+  </si>
+  <si>
+    <t>总大小（GB）</t>
+  </si>
+  <si>
+    <t>https://suche.transparenz.hamburg.de/dataset/3d-gebaeudemodell-lod1-de-hamburg2</t>
+  </si>
+  <si>
+    <t>.xml</t>
+  </si>
+  <si>
+    <t>https://3dbag.nl/en/</t>
+  </si>
+  <si>
+    <t>1.2，1.3</t>
+  </si>
+  <si>
+    <t>.json</t>
+  </si>
+  <si>
+    <t>7145 (28992)</t>
+  </si>
+  <si>
+    <t>数据质量不如lod2</t>
+  </si>
+  <si>
+    <t>https://opendata.dresden.de/informationsportal/#app/mainpage//3D%20Stadtmodell//</t>
+  </si>
+  <si>
+    <t>gml</t>
   </si>
   <si>
     <t>https://gdi.berlin.de/geonetwork/srv/ger/catalog.search#/metadata/e2a1e24e-bd9a-3de4-86af-af1a7a21a29e</t>
   </si>
   <si>
+    <t>json</t>
+  </si>
+  <si>
+    <t>https://data.public.lu/fr/datasets/batiments-3d-2013-lod-1-level-of-detail-1/</t>
+  </si>
+  <si>
+    <t>比lod2少不少，存在多栋建筑union一起的情况</t>
+  </si>
+  <si>
+    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/California.html</t>
+  </si>
+  <si>
+    <t>美国的数据无高程，ground_z是相对高度0</t>
+  </si>
+  <si>
+    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Illinois.html</t>
+  </si>
+  <si>
+    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Massachusetts.html</t>
+  </si>
+  <si>
+    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/DistrictofColumbia.html</t>
+  </si>
+  <si>
+    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/NewYork.html</t>
+  </si>
+  <si>
+    <t>曼哈顿</t>
+  </si>
+  <si>
+    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Oregon.html</t>
+  </si>
+  <si>
+    <t>https://front.geospatial.jp/plateau_portal_site/#</t>
+  </si>
+  <si>
+    <t>日本数据直接处理gml</t>
+  </si>
+  <si>
+    <t>Sapporo </t>
+  </si>
+  <si>
+    <t>https://www.geospatial.jp/ckan/dataset/plateau-01100-sapporo-shi-2020</t>
+  </si>
+  <si>
+    <t>https://www.geospatial.jp/ckan/dataset/plateau-27100-osaka-shi-2025</t>
+  </si>
+  <si>
+    <t>https://www.geospatial.jp/ckan/dataset/plateau-17201-kanazawa-shi-2024</t>
+  </si>
+  <si>
+    <t>https://open.toronto.ca/dataset/3d-massing/</t>
+  </si>
+  <si>
+    <t>shp</t>
+  </si>
+  <si>
+    <t>https://www.wien.gv.at/ma41datenviewer/public/</t>
+  </si>
+  <si>
+    <t>https://festudio.ca/research/buildings</t>
+  </si>
+  <si>
+    <t>https://github.com/AICyberTeam/GABLE</t>
+  </si>
+  <si>
+    <t>顶点过多，需要simplify，效果不好，失去形状</t>
+  </si>
+  <si>
+    <t>https://www.stadt-zuerich.ch/geodaten/download/Bauten___Blockmodell?format=10007</t>
+  </si>
+  <si>
+    <t>https://opendata.comune.bologna.it/explore/dataset/c_a944ctc_edifici_pl/export/?disjunctive.descrizion&amp;disjunctive.origine&amp;sort=-codice_ogg</t>
+  </si>
+  <si>
+    <t>geojson</t>
+  </si>
+  <si>
+    <t>https://www.data.gouv.fr/datasets/base-de-donnees-nationale-des-batiments</t>
+  </si>
+  <si>
+    <t>parquet</t>
+  </si>
+  <si>
+    <t>需要单独分离bbox</t>
+  </si>
+  <si>
+    <t>需要单独分离</t>
+  </si>
+  <si>
+    <t>surface count</t>
+  </si>
+  <si>
+    <t>https://suche.transparenz.hamburg.de/dataset/3d-gebaeudemodell-lod2-de-hamburg2</t>
+  </si>
+  <si>
     <t>xml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>building data source url</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>lod level</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>download time</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>format</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://suche.transparenz.hamburg.de/dataset/3d-gebaeudemodell-lod1-de-hamburg2</t>
-  </si>
-  <si>
-    <t>https://suche.transparenz.hamburg.de/dataset/3d-gebaeudemodell-lod2-de-hamburg2</t>
-  </si>
-  <si>
-    <t>data time</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>city</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>country</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Germany</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hamburg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Switzerland</t>
-  </si>
-  <si>
-    <t>Zurich</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Amsterdam</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Netherlands</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://3dbag.nl/en/</t>
-  </si>
-  <si>
-    <t>building count</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>surface count</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>包含lod1的block</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>包含lod2的block</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vienna</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>.xml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Austria</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1.2，1.3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>.json</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>original SRID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>匹配到的数量</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.wien.gv.at/ma41datenviewer/public/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Montreal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>https://donnees.montreal.ca/en/dataset/maquette-numerique-plateau-mont-royal-batiments-lod2-avec-textures?</t>
   </si>
   <si>
-    <t>gml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Canada</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>continent</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Europe</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>North America</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>980.23（包含港口海面）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>仅有部分区域</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>原始数据大小（GB）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>备注</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Zurich</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>gml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>json</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Luxembourg</t>
-  </si>
-  <si>
-    <t>Hannover</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.swisstopo.admin.ch/de/landschaftmodell-swissbuildings3d-3-0-beta#swissBUILDINGS3D-3.0-Beta---Download</t>
+  </si>
+  <si>
+    <t>https://data.public.lu/en/datasets/base-de-donnees-nationale-des-batiments-3d-2023/#</t>
   </si>
   <si>
     <t>https://www.hannover.de/Leben-in-der-Region-Hannover/Verwaltungen-Kommunen/Die-Verwaltung-der-Landeshauptstadt-Hannover/Dezernate-und-Fachbereiche-der-LHH/Stadtentwicklung-und-Bauen/Fachbereich-Planen-und-Stadtentwicklung/Geoinformation/Open-GeoData/3D-Stadtmodell-und-Gel%C3%A4ndemodell/Digitales-3D-Stadtmodell</t>
   </si>
   <si>
-    <t>Luxembourg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://data.public.lu/en/datasets/base-de-donnees-nationale-des-batiments-3d-2023/#</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Rotterdam </t>
-  </si>
-  <si>
-    <t>Linz</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Namur</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>https://geo.data.linz.gv.at/katalog/geodata/3d_geo_daten_lod2/</t>
   </si>
   <si>
     <t>https://data.namur.be/explore/dataset/namur-3d-batiments-textures-par-dalle-de-200m/table/?dataChart=eyJxdWVyaWVzIjpbeyJjb25maWciOnsiZGF0YXNldCI6Im5hbXVyLTNkLWJhdGltZW50cy10ZXh0dXJlcy1wYXItZGFsbGUtZGUtMjAwbSIsIm9wdGlvbnMiOnt9fSwiY2hhcnRzIjpbeyJhbGlnbk1vbnRoIjp0cnVlLCJ0eXBlIjoiY29sdW1uIiwiZnVuYyI6IkNPVU5UIiwic2NpZW50aWZpY0Rpc3BsYXkiOnRydWUsImNvbG9yIjoiIzAxMUY0OSJ9XSwieEF4aXMiOiJub20iLCJtYXhwb2ludHMiOjUwLCJzb3J0IjoiIn1dLCJ0aW1lc2NhbGUiOiIiLCJkaXNwbGF5TGVnZW5kIjp0cnVlLCJhbGlnbk1vbnRoIjp0cnVlfQ%3D%3D&amp;location=13,50.43269,4.86943&amp;basemap=jawg.streets</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://geo.data.linz.gv.at/katalog/geodata/3d_geo_daten_lod2/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Belgium</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Prague</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>通过法向量判断surface语义有bug</t>
   </si>
   <si>
     <t>https://geoportalpraha.cz/en/data-and-services/7e6316e95cfe4f36ae06bbfb687bf34b</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://gdi.berlin.de/geonetwork/srv/ger/catalog.search#/metadata/3c7c49af-00a4-3bcd-bc00-20e7f0f1b7bf</t>
+  </si>
+  <si>
+    <t>有ClosureSurface语义，但忽略</t>
+  </si>
+  <si>
+    <t>https://maps.nyc.gov/download/3dmodel/</t>
+  </si>
+  <si>
+    <t>单位是英尺，需要0.3048；分体块但是坡屋顶好像缺少</t>
   </si>
   <si>
     <t>https://geoportaal.maaamet.ee/eng/Download-3D-data-p837.html</t>
   </si>
   <si>
-    <t>Dresden</t>
-  </si>
-  <si>
-    <t>https://opendata.dresden.de/informationsportal/#app/mainpage//3D%20Stadtmodell//</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://gdi.berlin.de/geonetwork/srv/ger/catalog.search#/metadata/3c7c49af-00a4-3bcd-bc00-20e7f0f1b7bf</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>xml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Czech </t>
-  </si>
-  <si>
-    <t>总lod2 block</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>总lod1 block</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>总building</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>总surface</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>总有效building</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>城市数量</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>New York</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://maps.nyc.gov/download/3dmodel/</t>
-  </si>
-  <si>
-    <t>USA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>json</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>7145 (28992)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>单位是英尺，需要0.3048；分体块但是坡屋顶好像缺少</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>通过法向量判断surface语义有bug</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>总大小（GB）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>surface count（自建）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>简称</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DE_HH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AT_VI</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NL_AM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CA_MT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CH_ZU</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>LU_LU</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DE_HA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BE_NA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AT_LZ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CZ_PR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DE_DD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>US_NY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NL_RO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>数据质量不如lod2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>有ClosureSurface语义，但忽略</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Estonia</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.swisstopo.admin.ch/de/landschaftmodell-swissbuildings3d-3-0-beta#swissBUILDINGS3D-3.0-Beta---Download</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://data.public.lu/fr/datasets/batiments-3d-2013-lod-1-level-of-detail-1/</t>
-  </si>
-  <si>
-    <t>DE_BE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>比lod2少不少，存在多栋建筑union一起的情况</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/California.html</t>
-  </si>
-  <si>
-    <t>San Francisco</t>
-  </si>
-  <si>
-    <t>Chicago</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Boston</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Massachusetts.html</t>
-  </si>
-  <si>
-    <t>初始切片数量（仅排除&lt;1000）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>US_SF</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>US_CH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/DistrictofColumbia.html</t>
-  </si>
-  <si>
-    <t>US_WA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Washington D.C.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Portland</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/NewYork.html</t>
-  </si>
-  <si>
-    <t>http://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Oregon.html</t>
-  </si>
-  <si>
-    <t>美国的数据无高程，ground_z是相对高度0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>曼哈顿</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>US_BO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>US_PO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Tokyo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://front.geospatial.jp/plateau_portal_site/#</t>
-  </si>
-  <si>
-    <t>Sapporo </t>
-  </si>
-  <si>
-    <t>https://www.geospatial.jp/ckan/dataset/plateau-01100-sapporo-shi-2020</t>
-  </si>
-  <si>
-    <t>Asia</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Japan</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>42548.04（好多岛）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Sapporo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Osaka</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.geospatial.jp/ckan/dataset/plateau-27100-osaka-shi-2025</t>
-  </si>
-  <si>
-    <t>日本数据直接处理gml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.geospatial.jp/ckan/dataset/plateau-17201-kanazawa-shi-2024</t>
-  </si>
-  <si>
-    <t>Kanazawa</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JP_TK</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JP_SP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JP_OS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JP_KA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EE_TL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Tallinn</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>通过法向量判断surface语义有小bug，数据质量较差</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Toronto</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://open.toronto.ca/dataset/3d-massing/</t>
-  </si>
-  <si>
-    <t>shp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>data (update) time</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CA_TO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vienna</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.wien.gv.at/ma41datenviewer/public/</t>
-  </si>
-  <si>
-    <t>Winnipeg</t>
-  </si>
-  <si>
-    <t>https://festudio.ca/research/buildings</t>
-  </si>
-  <si>
-    <t>Munich</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>https://geodaten.bayern.de/opengeodata/OpenDataDetail.html?pn=lod2</t>
   </si>
   <si>
-    <t>DE_MU</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Nuremberg</t>
-  </si>
-  <si>
-    <t>CA_WP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DE_NU</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Winnipeg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Beijing</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Asia</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>China</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CN_BJ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>行政区域面积k㎡，只反应osm数据</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>shp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>顶点过多，需要simplify，效果不好，失去形状</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://github.com/AICyberTeam/GABLE</t>
-  </si>
-  <si>
-    <t>Bern</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.swisstopo.admin.ch/de/landschaftmodell-swissbuildings3d-3-0-beta#swissBUILDINGS3D-3.0-Beta---Download</t>
-  </si>
-  <si>
-    <t>gml</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>2021、2023</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CH_BE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Zurich</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.stadt-zuerich.ch/geodaten/download/Bauten___Blockmodell?format=10007</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>shp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://htmlpreview.github.io/?https://github.com/opencitymodel/opencitymodel/blob/master/releases/2019-jun/Illinois.html</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Bologna</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>geojson</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Italy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>IT_BO</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://opendata.comune.bologna.it/explore/dataset/c_a944ctc_edifici_pl/export/?disjunctive.descrizion&amp;disjunctive.origine&amp;sort=-codice_ogg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Lyon</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>https://data.grandlyon.com/portail/fr/jeux-de-donnees/maquettes-3d-texturees-2018-communes-metropole-lyon/donnees</t>
   </si>
   <si>
-    <t>France</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FR_LY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Paris</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FR_PA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>parquet</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.data.gouv.fr/datasets/base-de-donnees-nationale-des-batiments</t>
-  </si>
-  <si>
-    <t>需要单独分离</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Marseille</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FR_MA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>需要单独分离bbox</t>
+    <t xml:space="preserve"> </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -887,24 +693,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="15">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -919,7 +725,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -934,10 +740,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1259,71 +1065,78 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B6020B-322E-40F5-A134-4E53684558CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.4140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.9140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="1" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.08203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.9140625" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.08203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="9" style="1"/>
-    <col min="13" max="13" width="11.25" style="1" customWidth="1"/>
-    <col min="14" max="14" width="12.08203125" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="1"/>
+    <col min="6" max="6" width="15.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" style="1" customWidth="1"/>
+    <col min="8" max="9" width="9.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="9" style="1" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="12.109375" style="1" customWidth="1"/>
+    <col min="15" max="16" width="9" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="42" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="N1" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D2" s="3">
         <v>20260413</v>
@@ -1332,7 +1145,7 @@
         <v>20260413</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G2" s="3">
         <v>6538</v>
@@ -1344,8 +1157,12 @@
         <v>5162</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>82</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="K2" s="3">
+        <v>4899</v>
+      </c>
+      <c r="L2" s="3"/>
       <c r="M2" s="1">
         <f>SUM(H2:H50)</f>
         <v>261978</v>
@@ -1355,15 +1172,15 @@
         <v>79550</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D3" s="3">
         <v>20260417</v>
@@ -1384,18 +1201,21 @@
         <v>5871</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="K3" s="1">
+        <v>5700</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D4" s="3">
         <v>20260414</v>
@@ -1416,18 +1236,21 @@
         <v>3118</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="K4" s="1">
+        <v>2946</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1">
         <v>20260422</v>
@@ -1445,18 +1268,18 @@
         <v>1577</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D6" s="3">
         <v>20260414</v>
@@ -1477,18 +1300,21 @@
         <v>1319</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D7" s="4">
         <v>20260423</v>
@@ -1509,18 +1335,18 @@
         <v>507</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4">
         <v>20260423</v>
@@ -1538,18 +1364,18 @@
         <v>2000</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D9" s="3">
         <v>20260417</v>
@@ -1567,18 +1393,18 @@
         <v>926</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="D10" s="9">
         <v>20260424</v>
@@ -1596,18 +1422,18 @@
         <v>752</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="D11" s="1">
         <v>20260424</v>
@@ -1625,18 +1451,18 @@
         <v>4949</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1">
         <v>20260425</v>
@@ -1657,18 +1483,21 @@
         <v>2268</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="K12" s="1">
+        <v>2154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D13" s="10">
         <v>20260425</v>
@@ -1689,18 +1518,21 @@
         <v>28926</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+      <c r="K13" s="1">
+        <v>2598</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D14" s="1">
         <v>20260425</v>
@@ -1721,18 +1553,21 @@
         <v>2793</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="K14" s="1">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D15" s="1">
         <v>20260413</v>
@@ -1753,18 +1588,21 @@
         <v>9229</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="K15" s="1">
+        <v>8726</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D16" s="1">
         <v>20260427</v>
@@ -1782,18 +1620,21 @@
         <v>4732</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+      <c r="K16" s="1">
+        <v>4495</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D17" s="1">
         <v>20260427</v>
@@ -1811,18 +1652,21 @@
         <v>16898</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+      <c r="K17" s="1">
+        <v>16044</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D18" s="1">
         <v>20260427</v>
@@ -1840,18 +1684,21 @@
         <v>4015</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="K18" s="1">
+        <v>3803</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D19" s="1">
         <v>20260428</v>
@@ -1869,18 +1716,21 @@
         <v>4564</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="K19" s="1">
+        <v>4330</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="D20" s="1">
         <v>20260428</v>
@@ -1898,18 +1748,21 @@
         <v>9377</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+      <c r="K20" s="1">
+        <v>8902</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>124</v>
+        <v>64</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="D21" s="1">
         <v>20260428</v>
@@ -1918,7 +1771,7 @@
         <v>20260428</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="G21" s="1">
         <v>101419</v>
@@ -1927,18 +1780,21 @@
         <v>58668</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>124</v>
+        <v>64</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="D22" s="1">
         <v>20260428</v>
@@ -1956,18 +1812,21 @@
         <v>29955</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+      <c r="K22" s="1">
+        <v>28457</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>124</v>
+        <v>64</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="D23" s="1">
         <v>20260416</v>
@@ -1985,18 +1844,21 @@
         <v>23443</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+      <c r="K23" s="1">
+        <v>22265</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>132</v>
+        <v>72</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>124</v>
+        <v>64</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="D24" s="1">
         <v>20260429</v>
@@ -2014,18 +1876,21 @@
         <v>10052</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="K24" s="1">
+        <v>9549</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="D25" s="5">
         <v>20260424</v>
@@ -2044,18 +1909,20 @@
         <v>1119</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>140</v>
+        <v>77</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D26" s="1">
         <v>20260429</v>
@@ -2073,18 +1940,21 @@
         <v>10107</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+      <c r="K26" s="1">
+        <v>9594</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>155</v>
+        <v>79</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D27" s="1">
         <v>20260430</v>
@@ -2102,18 +1972,21 @@
         <v>5414</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+      <c r="K27" s="1">
+        <v>5142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D28" s="1">
         <v>20260430</v>
@@ -2132,18 +2005,20 @@
         <v>5085</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D29" s="1">
         <v>20260430</v>
@@ -2161,18 +2036,18 @@
         <v>1844</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>156</v>
+        <v>85</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>157</v>
+        <v>64</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>158</v>
+        <v>86</v>
       </c>
       <c r="D30" s="9">
         <v>20260504</v>
@@ -2191,18 +2066,20 @@
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>164</v>
+        <v>88</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D31" s="1">
         <v>20260414</v>
@@ -2220,18 +2097,18 @@
         <v>516</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>173</v>
+        <v>90</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>175</v>
+        <v>91</v>
       </c>
       <c r="D32" s="1">
         <v>20260507</v>
@@ -2249,18 +2126,21 @@
         <v>1204</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+      <c r="K32" s="1">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>178</v>
+        <v>93</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>180</v>
+        <v>94</v>
       </c>
       <c r="D33" s="1">
         <v>20260507</v>
@@ -2281,18 +2161,21 @@
         <v>1589</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+      <c r="K33" s="1">
+        <v>1511</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>182</v>
+        <v>96</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>180</v>
+        <v>94</v>
       </c>
       <c r="D34" s="1">
         <v>20260507</v>
@@ -2310,18 +2193,21 @@
         <v>3614</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+      <c r="K34" s="1">
+        <v>3431</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>180</v>
+        <v>94</v>
       </c>
       <c r="D35" s="1">
         <v>20260508</v>
@@ -2339,99 +2225,104 @@
         <v>2536</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>188</v>
+        <v>99</v>
+      </c>
+      <c r="K35" s="1">
+        <v>2409</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD8883F-BF25-46E4-9E09-E50E86F863DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.75" style="3" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="57.6640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="9" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.9140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="3" customWidth="1"/>
     <col min="5" max="5" width="11.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.08203125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14.08203125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.4140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="11.75" style="3" customWidth="1"/>
-    <col min="10" max="10" width="14.08203125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="11.75" style="3" customWidth="1"/>
-    <col min="12" max="12" width="23.9140625" style="3" customWidth="1"/>
-    <col min="13" max="15" width="9" style="3"/>
+    <col min="6" max="6" width="8.109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.77734375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="23.88671875" style="3" customWidth="1"/>
+    <col min="13" max="15" width="9" style="3" customWidth="1"/>
     <col min="16" max="16" width="11.6640625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="12.58203125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="11.08203125" style="3" customWidth="1"/>
-    <col min="19" max="16384" width="9" style="3"/>
+    <col min="17" max="17" width="12.5546875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="11.109375" style="3" customWidth="1"/>
+    <col min="19" max="20" width="9" style="3" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="42" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>29</v>
+        <v>107</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>30</v>
+        <v>108</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>42</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="M1"/>
       <c r="O1" s="12" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>70</v>
+        <v>114</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>116</v>
       </c>
       <c r="C2" s="3">
         <v>1</v>
@@ -2443,7 +2334,7 @@
         <v>20260414</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="G2" s="3">
         <v>384626</v>
@@ -2486,15 +2377,15 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>27</v>
+        <v>119</v>
       </c>
       <c r="D3" s="3">
         <v>20250903</v>
@@ -2503,7 +2394,7 @@
         <v>20260414</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>28</v>
+        <v>120</v>
       </c>
       <c r="G3" s="3">
         <v>165995</v>
@@ -2512,7 +2403,7 @@
         <v>1888041</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="J3" s="3">
         <v>150825</v>
@@ -2521,16 +2412,17 @@
         <v>1.01</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>95</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="M3"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="C4" s="3">
         <v>1</v>
@@ -2542,7 +2434,7 @@
         <v>20260424</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G4" s="3">
         <v>163530</v>
@@ -2559,13 +2451,14 @@
       <c r="K4" s="3">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+      <c r="M4"/>
+    </row>
+    <row r="5" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="C5" s="3">
         <v>1</v>
@@ -2577,7 +2470,7 @@
         <v>20260427</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G5" s="3">
         <v>928003</v>
@@ -2594,16 +2487,17 @@
       <c r="K5" s="3">
         <v>6.6</v>
       </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="M5"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>27</v>
+        <v>119</v>
       </c>
       <c r="D6" s="3">
         <v>20250903</v>
@@ -2612,7 +2506,7 @@
         <v>20260425</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G6" s="3">
         <v>189650</v>
@@ -2621,7 +2515,7 @@
         <v>1785785</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="J6" s="3">
         <v>154002</v>
@@ -2630,15 +2524,16 @@
         <v>1.04</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+      <c r="M6"/>
+    </row>
+    <row r="7" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -2650,7 +2545,7 @@
         <v>20260427</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G7" s="3">
         <v>10300</v>
@@ -2668,15 +2563,15 @@
         <v>0.05</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
@@ -2688,7 +2583,7 @@
         <v>20260427</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G8" s="3">
         <v>159456</v>
@@ -2706,15 +2601,16 @@
         <v>0.15</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+      <c r="M8"/>
+    </row>
+    <row r="9" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
       <c r="C9" s="3">
         <v>1</v>
@@ -2726,7 +2622,7 @@
         <v>20260427</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G9" s="3">
         <v>1617647</v>
@@ -2743,13 +2639,14 @@
       <c r="K9" s="3">
         <v>1.43</v>
       </c>
-    </row>
-    <row r="10" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+      <c r="M9"/>
+    </row>
+    <row r="10" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
@@ -2761,7 +2658,7 @@
         <v>20260427</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G10" s="3">
         <v>123192</v>
@@ -2778,13 +2675,14 @@
       <c r="K10" s="3">
         <v>0.11</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+      <c r="M10"/>
+    </row>
+    <row r="11" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="C11" s="3">
         <v>1</v>
@@ -2796,7 +2694,7 @@
         <v>20260428</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G11" s="3">
         <v>161911</v>
@@ -2813,6 +2711,7 @@
       <c r="K11" s="3">
         <v>0.19</v>
       </c>
+      <c r="M11"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
@@ -2820,12 +2719,12 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="40.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
@@ -2837,7 +2736,7 @@
         <v>20260428</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G12" s="3">
         <v>42974</v>
@@ -2855,15 +2754,16 @@
         <v>0.05</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" ht="42.65" customHeight="1" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+      <c r="M12"/>
+    </row>
+    <row r="13" spans="1:25" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="C13" s="3">
         <v>1</v>
@@ -2875,7 +2775,7 @@
         <v>20260428</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G13" s="3">
         <v>296701</v>
@@ -2892,13 +2792,14 @@
       <c r="K13" s="3">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="M13"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -2910,7 +2811,7 @@
         <v>20260428</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G14" s="3">
         <v>2005288</v>
@@ -2928,15 +2829,16 @@
         <v>31.3</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="28" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+      <c r="M14"/>
+    </row>
+    <row r="15" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
@@ -2948,7 +2850,7 @@
         <v>20260428</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G15" s="3">
         <v>646474</v>
@@ -2965,13 +2867,14 @@
       <c r="K15" s="3">
         <v>7.52</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="M15"/>
+    </row>
+    <row r="16" spans="1:25" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="C16" s="3">
         <v>1</v>
@@ -2983,7 +2886,7 @@
         <v>20260421</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G16" s="3">
         <v>616119</v>
@@ -3000,13 +2903,14 @@
       <c r="K16" s="3">
         <v>7.87</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+      <c r="M16"/>
+    </row>
+    <row r="17" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>132</v>
+        <v>72</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="C17" s="3">
         <v>1</v>
@@ -3018,7 +2922,7 @@
         <v>20260429</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G17" s="3">
         <v>213878</v>
@@ -3035,13 +2939,14 @@
       <c r="K17" s="3">
         <v>2.37</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M17"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>140</v>
+        <v>77</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C18" s="3">
         <v>1</v>
@@ -3053,7 +2958,7 @@
         <v>20260429</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G18" s="3">
         <v>409703</v>
@@ -3070,13 +2975,14 @@
       <c r="K18" s="3">
         <v>0.28999999999999998</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M18"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>146</v>
       </c>
       <c r="C19" s="3">
         <v>1.4</v>
@@ -3088,7 +2994,7 @@
         <v>20260429</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G19" s="3">
         <v>695635</v>
@@ -3105,13 +3011,14 @@
       <c r="K19" s="3">
         <v>0.26</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M19"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>147</v>
+        <v>79</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C20" s="3">
         <v>1</v>
@@ -3123,7 +3030,7 @@
         <v>20260430</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G20" s="3">
         <v>282398</v>
@@ -3140,13 +3047,14 @@
       <c r="K20" s="3">
         <v>0.28999999999999998</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+      <c r="M20"/>
+    </row>
+    <row r="21" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>156</v>
+        <v>85</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="C21" s="6">
         <v>1</v>
@@ -3158,7 +3066,7 @@
         <v>20260415</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="G21" s="6">
         <v>4088130</v>
@@ -3176,15 +3084,15 @@
         <v>1.79</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>169</v>
+        <v>29</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>170</v>
+        <v>149</v>
       </c>
       <c r="C22" s="3">
         <v>1</v>
@@ -3196,7 +3104,7 @@
         <v>20260506</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>171</v>
+        <v>144</v>
       </c>
       <c r="G22" s="3">
         <v>65986</v>
@@ -3213,13 +3121,14 @@
       <c r="K22" s="3">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+      <c r="M22"/>
+    </row>
+    <row r="23" spans="1:13" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>173</v>
+        <v>90</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>177</v>
+        <v>150</v>
       </c>
       <c r="C23" s="3">
         <v>1</v>
@@ -3231,7 +3140,7 @@
         <v>20260507</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>174</v>
+        <v>151</v>
       </c>
       <c r="G23" s="3">
         <v>54707</v>
@@ -3248,13 +3157,14 @@
       <c r="K23" s="3">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+      <c r="M23"/>
+    </row>
+    <row r="24" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>182</v>
+        <v>96</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="C24" s="3">
         <v>1</v>
@@ -3266,7 +3176,7 @@
         <v>20260508</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="G24" s="3">
         <v>86053</v>
@@ -3284,15 +3194,16 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+      <c r="M24"/>
+    </row>
+    <row r="25" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>178</v>
+        <v>93</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="C25" s="3">
         <v>1</v>
@@ -3304,7 +3215,7 @@
         <v>20260508</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="G25" s="3">
         <v>59983</v>
@@ -3322,15 +3233,16 @@
         <v>0.03</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+        <v>155</v>
+      </c>
+      <c r="M25"/>
+    </row>
+    <row r="26" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="C26" s="14">
         <v>1</v>
@@ -3342,7 +3254,7 @@
         <v>20260508</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="G26" s="14">
         <v>153114</v>
@@ -3360,105 +3272,107 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="L26" s="14" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.3"/>
+        <v>155</v>
+      </c>
+      <c r="M26"/>
+    </row>
+    <row r="27" spans="1:13" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B22" r:id="rId1" xr:uid="{0792EE3E-1FC9-4CAD-B9CA-7BF3E57258DA}"/>
-    <hyperlink ref="B9" r:id="rId2" xr:uid="{67BF9F36-3AB9-4878-BFBB-1333C799934B}"/>
-    <hyperlink ref="B23" r:id="rId3" xr:uid="{8B6B8B01-CB53-4746-9684-09463546D292}"/>
+    <hyperlink ref="B9" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B22" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="B23" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{830BA63A-35BF-480A-BCDB-E5D49BE645A6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:S20"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.75" style="3" customWidth="1"/>
-    <col min="2" max="2" width="76.9140625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="76.88671875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" style="3"/>
-    <col min="7" max="7" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.25" style="3" customWidth="1"/>
-    <col min="9" max="9" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.75" style="3" customWidth="1"/>
-    <col min="11" max="11" width="16.75" style="3" customWidth="1"/>
-    <col min="12" max="12" width="26.08203125" style="3" customWidth="1"/>
-    <col min="13" max="15" width="9" style="3"/>
-    <col min="16" max="16" width="11.4140625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="13.08203125" style="3" customWidth="1"/>
-    <col min="18" max="19" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="3"/>
+    <col min="6" max="6" width="9" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.21875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.77734375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.77734375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="26.109375" style="3" customWidth="1"/>
+    <col min="13" max="15" width="9" style="3" customWidth="1"/>
+    <col min="16" max="16" width="11.44140625" style="3" customWidth="1"/>
+    <col min="17" max="17" width="13.109375" style="3" customWidth="1"/>
+    <col min="18" max="19" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9" style="3" customWidth="1"/>
+    <col min="22" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>29</v>
+        <v>107</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>30</v>
+        <v>108</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>70</v>
+        <v>114</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="C2" s="3">
         <v>2</v>
@@ -3470,7 +3384,7 @@
         <v>20260414</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="G2" s="3">
         <v>388267</v>
@@ -3508,12 +3422,12 @@
         <v>86.720000000000013</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>31</v>
+        <v>145</v>
       </c>
       <c r="C3" s="3">
         <v>2.1</v>
@@ -3525,7 +3439,7 @@
         <v>20260416</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
       <c r="G3" s="3">
         <v>477126</v>
@@ -3543,12 +3457,12 @@
         <v>11.1</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="C4" s="3">
         <v>2.2000000000000002</v>
@@ -3560,7 +3474,7 @@
         <v>20260414</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>45</v>
+        <v>126</v>
       </c>
       <c r="G4" s="3">
         <v>165992</v>
@@ -3569,7 +3483,7 @@
         <v>3236008</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="J4" s="3">
         <v>146861</v>
@@ -3578,12 +3492,12 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>33</v>
+        <v>159</v>
       </c>
       <c r="C5" s="3">
         <v>2</v>
@@ -3595,7 +3509,7 @@
         <v>20260422</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
       <c r="G5" s="3">
         <v>37885</v>
@@ -3613,15 +3527,15 @@
         <v>3.7</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>98</v>
+        <v>161</v>
       </c>
       <c r="C6" s="3">
         <v>2</v>
@@ -3633,7 +3547,7 @@
         <v>20260414</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
       <c r="G6" s="3">
         <v>50600</v>
@@ -3651,12 +3565,12 @@
         <v>7.41</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>50</v>
+        <v>162</v>
       </c>
       <c r="C7" s="3">
         <v>2.2000000000000002</v>
@@ -3668,7 +3582,7 @@
         <v>20260423</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G7" s="3">
         <v>23275</v>
@@ -3686,12 +3600,12 @@
         <v>1.03</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="70" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>48</v>
+        <v>163</v>
       </c>
       <c r="C8" s="3">
         <v>2</v>
@@ -3703,7 +3617,7 @@
         <v>20260423</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G8" s="3">
         <v>135775</v>
@@ -3721,12 +3635,12 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="C9" s="3">
         <v>2</v>
@@ -3738,7 +3652,7 @@
         <v>20260424</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G9" s="3">
         <v>68529</v>
@@ -3756,12 +3670,12 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="98" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>54</v>
+        <v>165</v>
       </c>
       <c r="C10" s="6">
         <v>2.2000000000000002</v>
@@ -3773,7 +3687,7 @@
         <v>20260424</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G10" s="6">
         <v>63153</v>
@@ -3791,15 +3705,15 @@
         <v>1.08</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>58</v>
+        <v>167</v>
       </c>
       <c r="C11" s="3">
         <v>2</v>
@@ -3811,7 +3725,7 @@
         <v>20260424</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G11" s="3">
         <v>366007</v>
@@ -3829,12 +3743,12 @@
         <v>4.72</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="C12" s="3">
         <v>2</v>
@@ -3846,7 +3760,7 @@
         <v>20260424</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G12" s="3">
         <v>163576</v>
@@ -3864,12 +3778,12 @@
         <v>3.69</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>63</v>
+        <v>168</v>
       </c>
       <c r="C13" s="3">
         <v>2</v>
@@ -3881,7 +3795,7 @@
         <v>20260425</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>64</v>
+        <v>158</v>
       </c>
       <c r="G13" s="3">
         <v>874612</v>
@@ -3899,15 +3813,15 @@
         <v>14.3</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>73</v>
+        <v>170</v>
       </c>
       <c r="C14" s="11">
         <v>2</v>
@@ -3919,7 +3833,7 @@
         <v>20260425</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G14" s="11">
         <v>1083432</v>
@@ -3937,15 +3851,15 @@
         <v>12.8</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" s="11" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="C15" s="3">
         <v>2.2000000000000002</v>
@@ -3957,7 +3871,7 @@
         <v>20260425</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="G15" s="3">
         <v>189649</v>
@@ -3966,7 +3880,7 @@
         <v>2910029</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="J15" s="3">
         <v>154002</v>
@@ -3975,12 +3889,12 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>59</v>
+        <v>172</v>
       </c>
       <c r="C16" s="6">
         <v>2</v>
@@ -3992,7 +3906,7 @@
         <v>20260429</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G16" s="6">
         <v>49790</v>
@@ -4010,15 +3924,15 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="C17" s="3">
         <v>2</v>
@@ -4027,7 +3941,7 @@
         <v>20260430</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G17" s="3">
         <v>373913</v>
@@ -4045,12 +3959,12 @@
         <v>5.97</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
@@ -4059,7 +3973,7 @@
         <v>20260430</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="G18" s="3">
         <v>219925</v>
@@ -4077,24 +3991,24 @@
         <v>3.29</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="28" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>164</v>
+        <v>88</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E19" s="3">
         <v>20260506</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>166</v>
+        <v>124</v>
       </c>
       <c r="G19" s="3">
         <v>46569</v>
@@ -4112,12 +4026,12 @@
         <v>4.68</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="28" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>178</v>
+        <v>93</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C20" s="3">
         <v>2</v>
@@ -4129,7 +4043,7 @@
         <v>20260508</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>166</v>
+        <v>124</v>
       </c>
       <c r="G20" s="3">
         <v>24477</v>
@@ -4150,14 +4064,14 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{1D8E57E7-6951-45D0-9000-A48A5D2D54C6}"/>
-    <hyperlink ref="B7" r:id="rId2" xr:uid="{96022790-C32D-416D-A00B-0A4BF9F2B56B}"/>
-    <hyperlink ref="B10" r:id="rId3" display="https://data.namur.be/explore/dataset/namur-3d-batiments-textures-par-dalle-de-200m/table/?dataChart=eyJxdWVyaWVzIjpbeyJjb25maWciOnsiZGF0YXNldCI6Im5hbXVyLTNkLWJhdGltZW50cy10ZXh0dXJlcy1wYXItZGFsbGUtZGUtMjAwbSIsIm9wdGlvbnMiOnt9fSwiY2hhcnRzIjpbeyJhbGlnbk1vbnRoIjp0cnVlLCJ0eXBlIjoiY29sdW1uIiwiZnVuYyI6IkNPVU5UIiwic2NpZW50aWZpY0Rpc3BsYXkiOnRydWUsImNvbG9yIjoiIzAxMUY0OSJ9XSwieEF4aXMiOiJub20iLCJtYXhwb2ludHMiOjUwLCJzb3J0IjoiIn1dLCJ0aW1lc2NhbGUiOiIiLCJkaXNwbGF5TGVnZW5kIjp0cnVlLCJhbGlnbk1vbnRoIjp0cnVlfQ%3D%3D&amp;location=13,50.43269,4.86943&amp;basemap=jawg.streets" xr:uid="{94A87E04-C59B-4BD3-AF9B-9D043761E1D9}"/>
-    <hyperlink ref="B9" r:id="rId4" xr:uid="{8EB12734-1F40-4C6C-9742-A9BDC38D4641}"/>
-    <hyperlink ref="B11" r:id="rId5" xr:uid="{BDE7F4CE-843A-4272-8176-D2103C2BB35F}"/>
-    <hyperlink ref="B16" r:id="rId6" xr:uid="{A240AE20-DEEF-4E3D-99AF-D7289C26B140}"/>
-    <hyperlink ref="B13" r:id="rId7" location="/metadata/3c7c49af-00a4-3bcd-bc00-20e7f0f1b7bf" xr:uid="{BE79DDA7-5C97-4BFD-AC4A-EE3153109F0D}"/>
-    <hyperlink ref="B6" r:id="rId8" location="swissBUILDINGS3D-3.0-Beta---Download" xr:uid="{2AA2DC00-6403-4581-AA92-5AF06508077A}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="B6" r:id="rId2" location="swissBUILDINGS3D-3.0-Beta---Download" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="B9" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="B10" r:id="rId5" display="https://data.namur.be/explore/dataset/namur-3d-batiments-textures-par-dalle-de-200m/table/?dataChart=eyJxdWVyaWVzIjpbeyJjb25maWciOnsiZGF0YXNldCI6Im5hbXVyLTNkLWJhdGltZW50cy10ZXh0dXJlcy1wYXItZGFsbGUtZGUtMjAwbSIsIm9wdGlvbnMiOnt9fSwiY2hhcnRzIjpbeyJhbGlnbk1vbnRoIjp0cnVlLCJ0eXBlIjoiY29sdW1uIiwiZnVuYyI6IkNPVU5UIiwic2NpZW50aWZpY0Rpc3BsYXkiOnRydWUsImNvbG9yIjoiIzAxMUY0OSJ9XSwieEF4aXMiOiJub20iLCJtYXhwb2ludHMiOjUwLCJzb3J0IjoiIn1dLCJ0aW1lc2NhbGUiOiIiLCJkaXNwbGF5TGVnZW5kIjp0cnVlLCJhbGlnbk1vbnRoIjp0cnVlfQ%3D%3D&amp;location=13,50.43269,4.86943&amp;basemap=jawg.streets" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="B11" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="B13" r:id="rId7" location="/metadata/3c7c49af-00a4-3bcd-bc00-20e7f0f1b7bf" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="B16" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId9"/>

</xml_diff>